<commit_message>
Add the strong legacy PG answers to the SME packs as proposals
Put the strong evidence from the legacy O2C PG cross-comparison in
front of the SMEs, so they confirm or correct an answer instead of
writing one:

- Main pack: 11 questions (46 items). A1 gets a Legacy PG proposal
  column; A2 and A3 get one proposal for all 13 guides; A7, B3.1,
  B5.1, B5.2, B6, B7, B9 and B11 get a proposal paragraph.
- Part 2 supplement: 11 questions (16 items): P2-A1, A2, A3, B2, B4,
  B9, B10, C2, D2, E1 and E2.
- Both response sheets: a Legacy PG proposal column on Questions and a
  matching marker on Items. Answer cells stay empty.

Proposals are labelled as legacy reference evidence (D-044) and close
nothing on their own. Record the step as done in the cross-comparison,
the project notes and the README.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZin2KGg3LsvRGRgN9LWDp
</commit_message>
<xml_diff>
--- a/ar-collections-learning/03-validation/SME-Question-Pack-Part2-Responses.xlsx
+++ b/ar-collections-learning/03-validation/SME-Question-Pack-Part2-Responses.xlsx
@@ -11,9 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$1:$K$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Questions'!$A$1:$L$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Questions'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Items'!$A$1:$H$51</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Items'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -496,12 +496,13 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -532,30 +533,35 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Legacy PG proposal</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Answers items</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Blocking</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Answer</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Answered by</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Attachment or notes</t>
         </is>
@@ -589,16 +595,21 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>For CPJ-16: Post is on the Main toolbar. A journal that needs approval shows the Approval button and hides Post until it is approved; the journal is posted after approval. As partial evidence only, the legacy PGs have the Collections Officer prepare transfers between customer accounts and the Receipting Officer create manual payment journals. The security role (CPJ-21) is not covered. Source: 230 §6.7 steps 23 to 25 and Roles; 220 §4.1 steps 9 to 11 and Roles.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>GOV-01; CPJ-16; CPJ-21</t>
         </is>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -628,16 +639,21 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
+          <t>Christoper Clarke, the BPO on every version of the legacy Collections PG, which includes the transfer procedure (230 §6.7). The version history spells the name this way: please confirm the spelling. Source: 230 version history.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
           <t>GOV-02</t>
         </is>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -667,16 +683,21 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
+          <t>For CPJ-17: Yes. After Simulate posting, Approval &gt; Report as ready routes the journal. A user who is not an approver asks the Receipting team to approve it (Options &gt; Share &gt; Get a link gives a link to the journal). The approver clicks Approve, then the journal is posted. The journal name decides whether approval applies: "The journal name controls posting behavior and approval workflow." No value threshold is stated, and who authorizes a restoration (RO-03) is not covered. Source: 230 §6.7 steps 22 to 25; 220 §4.1 steps 5 and 9 to 11.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>CPJ-17; RO-03</t>
         </is>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="H4" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -704,18 +725,19 @@
           <t>Transfer: a payment posted to the wrong customer account, or funds to move to a confirmed related account. Distribution: a parent-account payment to distribute to confirmed child accounts. Restoration: an overpayment or written-off amount to put back on a customer account (the notes give no trigger).</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>TF-01; PC-06; RO-04</t>
         </is>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -743,18 +765,19 @@
           <t>Pending in all four documents.</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="n"/>
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>GOV-04</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="inlineStr"/>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -782,18 +805,19 @@
           <t>Not assigned.</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="n"/>
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>GOV-05</t>
         </is>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="2" t="inlineStr"/>
       <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -821,18 +845,19 @@
           <t>Notes: the current date is the default. Transfer notes: the original payment date "when appropriate". Restoration notes: a prior-period date only when required and the period is open. The parent-payment notes give no date rule.</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>CPJ-05</t>
         </is>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H8" s="2" t="inlineStr"/>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -862,16 +887,21 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
+          <t>Currency fills in from the line's Account. Confirm it matches the currency of the original receipt. If the currencies differ, stop and escalate before going on. Source: 230 §6.7 steps 12 and 19; 220 §4.2 step 9.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
           <t>CPJ-07</t>
         </is>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="2" t="inlineStr"/>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -899,18 +929,19 @@
           <t>Examples only: "Transfer funds from customer A to customer B"; "Overpayment put back on customer account".</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="n"/>
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>CPJ-04</t>
         </is>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="2" t="inlineStr"/>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -940,16 +971,21 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
+          <t>For TF-03: The legacy transfer procedure sets the source line's Offset account type to Ledger and its Offset account to 100949, "to ensure no impact to the bank". It does not give the account's name. Its destination line uses Bank instead, which contradicts this (see P2-C3). The Overpayment ledger (RO-01) is not covered. Source: 230 §6.7 steps 13 to 14 and 20 to 21.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>TF-03; RO-01</t>
         </is>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="2" t="inlineStr"/>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -977,18 +1013,19 @@
           <t>The notes state both rules for restoration entries only. The Restore guide applies them; the two transfer guides ask the question.</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>CPJ-10; CPJ-11</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="2" t="inlineStr"/>
       <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1016,18 +1053,19 @@
           <t>The transfer guide makes these prerequisites and puts the last two outside its scope until confirmed.</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="n"/>
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>TF-02; TF-05; TF-06</t>
         </is>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
       <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1055,18 +1093,19 @@
           <t>Part 1 notes: D365 has no reliable parent-child indicator; do not rely on account names. Notes: confirm from remittance, customer confirmation or other validated evidence; leave the residual on the parent with a note.</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="n"/>
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>PC-01; PC-02; PC-04; PC-05</t>
         </is>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="H14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1094,18 +1133,19 @@
           <t>The Restore guide covers both with one entry: a customer credit offset to the Overpayment ledger. Write-off processing is a separate backlog item (ranks 18 to 20).</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>RO-02</t>
         </is>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="H15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1135,16 +1175,21 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
+          <t>For CPJ-19: To reverse a posted journal: Accounts receivable &gt; Payments &gt; Customer payment journals, open the journal batch, select the payment line, click Voucher, then Reverse transactions. Set Use existing date for reversal (Yes keeps the original posting date) or enter a Reversal date, and enter a Reason comment. Click Reverse, then Post. Checking the result (CPJ-18) and unposted journals (CPJ-20) are not covered. Source: 220 §4.3.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
           <t>CPJ-18; CPJ-19; CPJ-20</t>
         </is>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="H16" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
       <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1174,16 +1219,21 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
+          <t>For SRC-03: Yes. The legacy PGs list AVA - Atlas Virtual Assistant, "your AI assistant for navigating the Procedure Guides", and the Procedure Guides as self-service resources. Simulate Posting errors (CPJ-15) are covered only as "a journal does not post while approval is pending or a validation error remains". Source: 230 and 200 Additional Resources; 220 Troubleshooting.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
           <t>CPJ-15; SRC-03</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n">
+      <c r="H17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H17" s="2" t="inlineStr"/>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1211,18 +1261,19 @@
           <t>Every step comes from Teams AI-generated notes. The step-evidence table in each guide preview shows the source of each step.</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="n"/>
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>SRC-01</t>
         </is>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="H18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1252,16 +1303,21 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
+          <t>For CPJ-01, CPJ-02, CPJ-03, CPJ-14: (Check against the recording.) +New creates the journal header. The journal name is selected in the Name field (CPJL, journal type Customer payments). The header Description fills in and is overwritten with the purpose. The Journal batch number hyperlink opens the lines, and +New adds a line, which has its own Description. Simulate Posting is Validate &gt; Simulate posting on the Main toolbar; errors appear as messages to correct before validating again. The legacy menu path is Accounts receivable &gt; Payments &gt; Customer payment journal(s), not Credit and collections as in the guides, so check both. Source: 230 §6.7 steps 3 to 17 and 22; 220 §4.1 steps 3 to 8.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
           <t>CPJ-01; CPJ-02; CPJ-03; CPJ-14</t>
         </is>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="H19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1289,18 +1345,19 @@
           <t>The guides apply the offset to every line, as the pack drafts imply.</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>CPJ-12; TF-04; PC-03</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n">
+      <c r="H20" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1328,18 +1385,19 @@
           <t>Not supplied.</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="n"/>
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>SRC-02</t>
         </is>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="H21" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="2" t="inlineStr"/>
       <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1367,18 +1425,19 @@
           <t>Working process names: AR Collections Customer Account Transfers, Parent Payment Distribution, Overpayment and Write-Off Restoration, and Customer Payment Journal Controls.</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>GOV-03</t>
         </is>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="H22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="2" t="inlineStr"/>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr"/>
+      <c r="L22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1408,16 +1467,21 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
+          <t>The legacy Collections PG prints the account number (100949) in its transfer steps, so the legacy precedent is to show account numbers. Source: 230 §6.7 step 14.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
           <t>CPJ-09</t>
         </is>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="H23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1445,18 +1509,19 @@
           <t>Proposed in D-036.</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="n"/>
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>SRC-04</t>
         </is>
       </c>
-      <c r="G24" s="2" t="n">
+      <c r="H24" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="2" t="inlineStr"/>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1486,16 +1551,21 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
+          <t>Yes. The legacy Collections PG v2.3 (October 2026) has a Customer Pools topic. Pools group customer accounts by defined criteria (customer group, legal entity or financial dimensions) and are assigned to Collections agents, to establish customer ownership and support follow-up and workload allocation. Managers (the Group Billing and Credit Manager) create and maintain the pools and the agent assignments. Source: 230 §3 and Roles.</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
           <t>CP-01; CP-02; CP-03</t>
         </is>
       </c>
-      <c r="G25" s="2" t="n">
+      <c r="H25" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="2" t="inlineStr"/>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1525,16 +1595,21 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
+          <t>For CP-04: A pool's criteria decide which customers it holds: Credit and collections &gt; Setup &gt; Customer pools, New, enter the Pool ID and Pool description, set Pool type = Collections, then Select pool criteria (Advanced query, Range tab: Table, Field, Criteria), Preview pool customers and Save. Pools reach a user through Credit and collections &gt; Setup &gt; Collections agents: add the Worker, add each Pool ID and set the Default pool. How pools change the daily work list (CP-06) is stated only as "ownership and workload allocation". Source: 230 §3.1 and §3.2.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
           <t>CP-04; CP-06</t>
         </is>
       </c>
-      <c r="G26" s="2" t="n">
+      <c r="H26" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="H26" s="2" t="inlineStr"/>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1562,18 +1637,19 @@
           <t>Not demonstrated in Part 1 or Part 2.</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="n"/>
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>CP-05</t>
         </is>
       </c>
-      <c r="G27" s="2" t="n">
+      <c r="H27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="2" t="inlineStr"/>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1601,21 +1677,22 @@
           <t>Kept as a validation backlog item only (D-035).</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="n"/>
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>CP-07</t>
         </is>
       </c>
-      <c r="G28" s="2" t="n">
+      <c r="H28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H28" s="2" t="inlineStr"/>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K28"/>
+  <autoFilter ref="A1:L28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
@@ -1627,7 +1704,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1637,6 +1714,7 @@
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1675,6 +1753,11 @@
           <t>Closed (Yes / No / Partly)</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Legacy PG proposal</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1708,6 +1791,7 @@
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1741,6 +1825,7 @@
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1774,6 +1859,11 @@
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1807,6 +1897,7 @@
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1840,6 +1931,7 @@
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1873,6 +1965,11 @@
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1906,6 +2003,7 @@
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1939,6 +2037,7 @@
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1972,6 +2071,7 @@
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2005,6 +2105,11 @@
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2038,6 +2143,11 @@
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2071,6 +2181,11 @@
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -2104,6 +2219,7 @@
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -2137,6 +2253,7 @@
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -2170,6 +2287,11 @@
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2203,6 +2325,11 @@
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2236,6 +2363,7 @@
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2269,6 +2397,7 @@
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2302,6 +2431,7 @@
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2335,6 +2465,11 @@
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2368,6 +2503,7 @@
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2401,6 +2537,11 @@
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2434,6 +2575,11 @@
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2467,6 +2613,7 @@
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
+      <c r="H25" s="2" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2500,6 +2647,11 @@
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2533,6 +2685,7 @@
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
+      <c r="H27" s="2" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2566,6 +2719,7 @@
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
+      <c r="H28" s="2" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2599,6 +2753,7 @@
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
+      <c r="H29" s="2" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2632,6 +2787,7 @@
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
+      <c r="H30" s="2" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2665,6 +2821,11 @@
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2698,6 +2859,7 @@
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
+      <c r="H32" s="2" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2731,6 +2893,7 @@
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2764,6 +2927,7 @@
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr"/>
+      <c r="H34" s="2" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2797,6 +2961,7 @@
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2830,6 +2995,7 @@
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr"/>
+      <c r="H36" s="2" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2863,6 +3029,7 @@
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr"/>
+      <c r="H37" s="2" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2896,6 +3063,7 @@
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr"/>
+      <c r="H38" s="2" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2929,6 +3097,7 @@
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr"/>
+      <c r="H39" s="2" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2962,6 +3131,7 @@
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr"/>
+      <c r="H40" s="2" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2995,6 +3165,7 @@
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr"/>
+      <c r="H41" s="2" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3028,6 +3199,7 @@
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr"/>
+      <c r="H42" s="2" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3061,6 +3233,7 @@
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3094,6 +3267,7 @@
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3127,6 +3301,11 @@
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3160,6 +3339,11 @@
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3193,6 +3377,11 @@
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3226,6 +3415,11 @@
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3259,6 +3453,7 @@
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3292,6 +3487,7 @@
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3325,9 +3521,10 @@
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G51"/>
+  <autoFilter ref="A1:H51"/>
   <dataValidations count="1">
     <dataValidation sqref="G2 G3 G4 G5 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 G21 G22 G23 G24 G25 G26 G27 G28 G29 G30 G31 G32 G33 G34 G35 G36 G37 G38 G39 G40 G41 G42 G43 G44 G45 G46 G47 G48 G49 G50 G51" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Partly"</formula1>

</xml_diff>